<commit_message>
budget keeper updated with loading txt data
</commit_message>
<xml_diff>
--- a/data/output/flood_report.xlsx
+++ b/data/output/flood_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,20 +436,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>province</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>flood_level_meters</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>vicm_count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>main_need</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -461,18 +466,23 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>9.5</v>
       </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -484,16 +494,21 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -505,16 +520,21 @@
           <t>Kandy</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -526,16 +546,21 @@
           <t>Kalutara</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -547,18 +572,23 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>2</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>500</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Food/Water</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -570,16 +600,21 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -591,16 +626,21 @@
           <t>Matara</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Southern</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -612,18 +652,23 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>1.5</v>
       </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -635,16 +680,21 @@
           <t>Galle</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Southern</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>0</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -656,16 +706,21 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
@@ -677,37 +732,39 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="n">
-        <v>40</v>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Colombo</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr"/>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Food/Water</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -719,16 +776,21 @@
           <t>Kandy</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -740,16 +802,21 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="n">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
         <v>200</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Food/Water</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -761,16 +828,21 @@
           <t>Nuwara Eliya</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>0</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -782,16 +854,21 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -803,18 +880,23 @@
           <t>Ratnapura</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sabaragamuwa</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
         <v>5</v>
       </c>
-      <c r="C18" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="D18" t="n">
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Warning</t>
         </is>
@@ -826,16 +908,21 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>0</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -847,18 +934,23 @@
           <t>Kalutara</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>0</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Warning</t>
         </is>
       </c>
     </row>
@@ -868,16 +960,21 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -889,16 +986,21 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Generator Fuel</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -910,18 +1012,23 @@
           <t>Kandy</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="D23" t="n">
+        <v>0</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -933,18 +1040,23 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>0</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Stable</t>
         </is>
       </c>
     </row>
@@ -954,16 +1066,21 @@
           <t>Kalutara</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="n">
-        <v>8</v>
-      </c>
-      <c r="D25" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -975,16 +1092,21 @@
           <t>Matara</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Southern</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -996,16 +1118,21 @@
           <t>Colombo</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="n">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="n">
         <v>5000</v>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
-      </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1017,16 +1144,21 @@
           <t>Galle</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Southern</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
@@ -1038,37 +1170,43 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="n">
-        <v>2</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>General Assistance</t>
-        </is>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Colombo</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Food/Water</t>
-        </is>
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>General Assistance</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1080,16 +1218,21 @@
           <t>Kegalle</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="n">
-        <v>10</v>
-      </c>
-      <c r="D31" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Western</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>Rescue</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>

</xml_diff>

<commit_message>
log llm output and saved as csv
</commit_message>
<xml_diff>
--- a/data/output/flood_report.xlsx
+++ b/data/output/flood_report.xlsx
@@ -706,11 +706,7 @@
           <t>Gampaha</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Western</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>0</v>
@@ -1035,16 +1031,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Gampaha</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Western</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
         <v>0</v>
@@ -1186,7 +1174,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Warning</t>
         </is>
       </c>
     </row>

</xml_diff>